<commit_message>
Update Nguyen Nhat Tuong Vy AI_log.xlsx
</commit_message>
<xml_diff>
--- a/AI_Audit_Log/Nguyen Nhat Tuong Vy AI_log.xlsx
+++ b/AI_Audit_Log/Nguyen Nhat Tuong Vy AI_log.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Tuong Vy\Documents\GitHub\Group1-LAB211\AI_Audit_Log\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Tuong Vy\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D1F82CE-50EE-42B3-907C-B73178BDD3FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE38AE11-C280-4F9B-89ED-1691DFFED555}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="20376" windowHeight="12096" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1. Metadata &amp; Summary" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="176">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="291" uniqueCount="238">
   <si>
     <t>AI AUDIT LOG - METADATA &amp; SUMMARY</t>
   </si>
@@ -91,12 +91,6 @@
     <t>GitHub Copilot</t>
   </si>
   <si>
-    <t>Auto-completion</t>
-  </si>
-  <si>
-    <t>Speed up coding</t>
-  </si>
-  <si>
     <t>[Add more...]</t>
   </si>
   <si>
@@ -163,27 +157,18 @@
     <t>DECISION</t>
   </si>
   <si>
-    <t>Screenshot comparison 10 vs 5</t>
-  </si>
-  <si>
     <t>002</t>
   </si>
   <si>
     <t>PROBLEM-SOLVING</t>
   </si>
   <si>
-    <t>Code snippet + timing comparison</t>
-  </si>
-  <si>
     <t>003</t>
   </si>
   <si>
     <t>VERIFICATION</t>
   </si>
   <si>
-    <t>Google Scholar screenshot</t>
-  </si>
-  <si>
     <t>HALLUCINATION DETECTION LOG (BẮT BUỘC)</t>
   </si>
   <si>
@@ -388,21 +373,6 @@
     <t>Employee Payroll Management Simulation</t>
   </si>
   <si>
-    <t>~95</t>
-  </si>
-  <si>
-    <t>Used to understand CSV schema design and Java file handling.”</t>
-  </si>
-  <si>
-    <t>Use AI to design a 7 CSV file schema and prepare a presentation for the topic Employee Salary Management.</t>
-  </si>
-  <si>
-    <t>“Understand payroll schema and Java CSV handling.”</t>
-  </si>
-  <si>
-    <t>AI helps design the schema of 7 CSV files, explains the concept of FK, race conditions and presentation instructions.</t>
-  </si>
-  <si>
     <t>Database Design</t>
   </si>
   <si>
@@ -478,80 +448,295 @@
     <t>Removed unsupported leave types and kept only required enum values</t>
   </si>
   <si>
+    <t>LeaveBalance Repository</t>
+  </si>
+  <si>
+    <t>Generate a Java LeaveBalanceRepository with add(), findByEmployeeId(), and getAll() methods.</t>
+  </si>
+  <si>
+    <t>AI generated a repository using an ArrayList with methods to add records, search by employee ID, and retrieve all leave balances.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: Reviewed repository methods and verified they satisfy project requirements. Contextualization: Repository only needs basic CRUD for current milestone. Creative Synthesis: Simplified the implementation to match the existing repository structure used in the project. Decision: Adopted the final repository implementation and confirmed functionality through unit tests.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Need to implement a repository to manage LeaveBalance objects in memory and support employee lookup.   </t>
+  </si>
+  <si>
+    <t>Repository Unit Test</t>
+  </si>
+  <si>
+    <t>Need to verify that LeaveBalanceRepository correctly stores and retrieves leave balance data</t>
+  </si>
+  <si>
+    <t>Generate JUnit tests for LeaveBalanceRepository methods.</t>
+  </si>
+  <si>
+    <t>AI generated test cases for add(), findByEmployeeId(), and getAll().</t>
+  </si>
+  <si>
+    <t>Critical Thinking: Reviewed expected outputs and compared them with actual results. Contextualization: Added representative test data for multiple employees. Creative Synthesis: Adjusted assertions to match repository behavior. Decision: All repository tests passed successfully.</t>
+  </si>
+  <si>
+    <t>Employee Controller</t>
+  </si>
+  <si>
+    <t>Need to implement EmployeeController to wrap repository methods for employee management.</t>
+  </si>
+  <si>
+    <t>Generate an EmployeeController that uses EmployeeRepository methods such as findById(), findByDeptId(), add(), update(), and delete().</t>
+  </si>
+  <si>
+    <t>AI suggested a controller structure that delegates CRUD operations to EmployeeRepository.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: Reviewed the controller design to ensure no business logic was placed in the controller. Contextualization: The controller should only coordinate between the View and Repository layers. Creative Synthesis: Adjusted method names and coding style to match the project. Decision: Implemented the final EmployeeController.</t>
+  </si>
+  <si>
+    <t>Need to verify that EmployeeController correctly interacts with EmployeeRepository.</t>
+  </si>
+  <si>
+    <t>Generate JUnit test cases for EmployeeController CRUD operations.</t>
+  </si>
+  <si>
+    <t>AI generated test scenarios for add, update, delete, and search operations.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: Compared expected and actual repository data after each operation. Contextualization: Tested normal CRUD cases using sample employee records. Creative Synthesis: Simplified assertions to fit project requirements. Decision: All controller tests passed successfully.</t>
+  </si>
+  <si>
+    <t>Employee View</t>
+  </si>
+  <si>
+    <t>Report View</t>
+  </si>
+  <si>
+    <t>Need to implement a console-based EmployeeView to perform employee CRUD operations through EmployeeController.</t>
+  </si>
+  <si>
+    <t>Need to create a ReportView to display payroll statistics in the console.</t>
+  </si>
+  <si>
+    <t>Generate a Java console EmployeeView that supports Create, Read, Update, and Delete operations using EmployeeController.</t>
+  </si>
+  <si>
+    <t>Generate a Java ReportView that displays total net salary, number of processed employees, and approved leave requests.</t>
+  </si>
+  <si>
+    <t>AI suggested a menu-driven console interface with CRUD options and controller method calls.</t>
+  </si>
+  <si>
+    <t>AI generated a report layout and suggested methods to retrieve summary information from the Controller.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: Reviewed the menu structure to ensure the View only handled user input and output. Contextualization: Business logic remained inside the Controller layer. Creative Synthesis: Modified prompts, menu layout, and validation to match the project requirements. Decision: Completed the EmployeeView implementation.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: Verified that all report data came from the Controller instead of the View. Contextualization: The report summarizes payroll and leave information after processing. Creative Synthesis: Adjusted the output format to improve readability. Decision: Implemented the final ReportView successfully.</t>
+  </si>
+  <si>
     <t>004</t>
   </si>
   <si>
     <t>005</t>
   </si>
   <si>
-    <t>LeaveBalance Repository</t>
-  </si>
-  <si>
-    <t>Need a repository to manage leave balance records stored in CSV files</t>
-  </si>
-  <si>
-    <t>Generate a simple LeaveBalanceRepository class for Java CSV-based payroll system</t>
-  </si>
-  <si>
-    <t>AI suggested repository methods such as add(), findByEmployeeId(), and getAll()</t>
-  </si>
-  <si>
-    <t>AI suggested extending Exception and creating a custom constructor</t>
-  </si>
-  <si>
-    <t>AI suggested extending Exception with a message constructor</t>
-  </si>
-  <si>
-    <t>Create a custom InsufficientLeaveException in Java</t>
-  </si>
-  <si>
-    <t>Create a CsvParseException class for Java CSV processing</t>
-  </si>
-  <si>
-    <t>Critical Thinking: Reviewed repository methods. Contextualization: Project stores data in CSV instead of a database. Creative Synthesis: Simplified repository structure to match project requirements. Decision: Implemented LeaveBalanceRepository with basic operations.</t>
-  </si>
-  <si>
-    <t>Critical Thinking: Evaluated whether custom exception improves readability. Contextualization: Leave requests must validate available leave balance. Creative Synthesis: Integrated exception into leave validation logic. Decision: Implemented InsufficientLeaveException.</t>
-  </si>
-  <si>
-    <t>Critical Thinking: Verified that CSV parsing errors should be handled separately. Contextualization: CSV is the project's primary data storage format. Creative Synthesis: Used a dedicated exception for CSV validation errors. Decision: Implemented CsvParseException for parsing failures.</t>
-  </si>
-  <si>
     <t>006</t>
   </si>
   <si>
     <t>007</t>
   </si>
   <si>
-    <t>Exception Handling</t>
-  </si>
-  <si>
-    <t>CSV Validation</t>
-  </si>
-  <si>
-    <t>Need a custom exception when employees request more leave than available</t>
-  </si>
-  <si>
-    <t>Need a custom exception for invalid CSV data parsing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-</t>
-  </si>
-  <si>
-    <t>Overengineering</t>
-  </si>
-  <si>
-    <t>AI suggested database-oriented repository methods and complex persistence logic</t>
-  </si>
-  <si>
-    <t>Project only requires simple CSV-based storage and retrieval</t>
-  </si>
-  <si>
-    <t>Compared AI output with project requirements and existing architecture</t>
-  </si>
-  <si>
-    <t>Simplified repository implementation to basic CSV operations</t>
+    <t>008</t>
+  </si>
+  <si>
+    <t>009</t>
+  </si>
+  <si>
+    <t>010</t>
+  </si>
+  <si>
+    <t xml:space="preserve">005 </t>
+  </si>
+  <si>
+    <t>AI generated additional repository methods such as update(),delete(),and findAll() for LeaveBalanceRepository</t>
+  </si>
+  <si>
+    <t>The project milestone only required add (),findByEmployeeId(), and getAll().</t>
+  </si>
+  <si>
+    <t>Compared the generated code with the Week 4 repository requirements and existing implementation.</t>
+  </si>
+  <si>
+    <t>Removed unnecessary methods and kept only the required repository functions.</t>
+  </si>
+  <si>
+    <t>Code Generation Error</t>
+  </si>
+  <si>
+    <t>AI generated Junit test cases using methods that did not exist in the LeaveBalanceRepository.</t>
+  </si>
+  <si>
+    <t>The generated tests failed because those methods did not exist.</t>
+  </si>
+  <si>
+    <t>Executed the generated tests and compared them with the actual repository source code.</t>
+  </si>
+  <si>
+    <t>Updated the unit tests to match the implemented repository methods and verified all tests passed.</t>
+  </si>
+  <si>
+    <t>AI generated EmployeeController with business logic beyond the required CRUD wrapper methods.</t>
+  </si>
+  <si>
+    <t>The project specification only required EmployeeController to wrap EmployeeRepository methods and coordinate MVC flow.</t>
+  </si>
+  <si>
+    <t>Compared the AI-generated controller with the Week 5 task description and repository implementation.</t>
+  </si>
+  <si>
+    <t>Simplified EmployeeController to include only the required CRUD wrapper methods.</t>
+  </si>
+  <si>
+    <t>AI suggested handling employee management logic directly inside EmployeeView.</t>
+  </si>
+  <si>
+    <t>According to the project's MVC architecture, EmployeeView should only manage user input/output while EmployeeController handles business logic.</t>
+  </si>
+  <si>
+    <t>Reviewed the MVC design and compared it with the AI-generated code.</t>
+  </si>
+  <si>
+    <t>Moved business logic from EmployeeView to EmployeeController and kept the View responsible only for console interaction.</t>
+  </si>
+  <si>
+    <t>011</t>
+  </si>
+  <si>
+    <t>Synchronization (NO_LOCK)</t>
+  </si>
+  <si>
+    <t>Need to implement NO_LOCK synchronization mechanism for payroll simulation.</t>
+  </si>
+  <si>
+    <t>Explain how to implement a NO_LOCK synchronization mechanism in Java for payroll processing.</t>
+  </si>
+  <si>
+    <t>AI explained the concept of NO_LOCK and suggested a simple multithreaded implementation without synchronization.</t>
+  </si>
+  <si>
+    <t>ReportView Integration</t>
+  </si>
+  <si>
+    <t>Need to display payroll,employee and attendance reports through MVC.</t>
+  </si>
+  <si>
+    <t>Generate a ReportView that communicates with Controller instead of Repository.</t>
+  </si>
+  <si>
+    <t>AI generated a ReportView following the MVC pattern with report functions.</t>
+  </si>
+  <si>
+    <t>Main System Integration</t>
+  </si>
+  <si>
+    <t>Need to integrate all completed modules into the main application.</t>
+  </si>
+  <si>
+    <t>How should MainView organize different functional modules in an MVC payroll system?</t>
+  </si>
+  <si>
+    <t>AI suggested a menu-based architecture that initializes each View and Controller through dependency injection.</t>
+  </si>
+  <si>
+    <t>System Testing &amp; Demo</t>
+  </si>
+  <si>
+    <t>Need to verify that all functions work correctly before the final demonstration.</t>
+  </si>
+  <si>
+    <t>Provide a checklist for testing an Employee Payroll Management Simulation System.</t>
+  </si>
+  <si>
+    <t>AI suggested testing CRUD operations, payroll processing, leave requests, reports and synchronization mechanisms.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: Verified that the implementation intentionally allows race conditions. Contextualization: NO_LOCK is used only for comparison experiments, not production. Creative Synthesis: Adapted the code to fit the project architecture and simulator. Decision: Implemented NO_LOCK as the baseline mechanism.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: Removed unnecessary methods and adjusted menu options. Contextualization: The project requires View → Controller communication only. Creative Synthesis: Integrated ReportView into MainView and tested report functions. Decision: Used the modified ReportView in the final project.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: Simplified object creation to match the existing project. Contextualization: Integration must not change module responsibilities. Creative Synthesis: Connected Employee, Leave, Attendance, Payroll and Report modules into MainView. Decision: Finalized the integrated application structure.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: Executed only the test cases required by the project. Contextualization: Compared actual outputs with expected results. Creative Synthesis: Fixed minor integration issues before demo. Decision: Completed the final system testing successfully</t>
+  </si>
+  <si>
+    <t>012</t>
+  </si>
+  <si>
+    <t>013</t>
+  </si>
+  <si>
+    <t>014</t>
+  </si>
+  <si>
+    <t>015</t>
+  </si>
+  <si>
+    <t>Flowchart Design</t>
+  </si>
+  <si>
+    <t>Need to create flowcharts from Use Case Diagram and Class Diagram for the project report.</t>
+  </si>
+  <si>
+    <t>Create flowcharts for Employee Payroll Management System based on the Use Case Diagram and Class Diagram.</t>
+  </si>
+  <si>
+    <t>AI generated flowchart structures for Employee Management, Leave Management, Payroll Processing and Report modules, showing the processing sequence and decision points.</t>
+  </si>
+  <si>
+    <t>AI suggested that NO_LOCK should prevent duplicate payroll entries automatically.</t>
+  </si>
+  <si>
+    <t>NO_LOCK intentionally performs no synchronization, so race conditions and duplicate payments are expected.</t>
+  </si>
+  <si>
+    <t>Compared AI explanation with project synchronization requirements and experiment results.</t>
+  </si>
+  <si>
+    <t>Implemented NO_LOCK without synchronization and used it only as the baseline mechanism for comparison.</t>
+  </si>
+  <si>
+    <t>AI generated a flowchart that did not fully match the implemented MVC workflow.</t>
+  </si>
+  <si>
+    <t>The project flow requires View → Controller → Repository communication only.</t>
+  </si>
+  <si>
+    <t>Compared the AI-generated flowchart with the Use Case Diagram, Class Diagram, and source code.</t>
+  </si>
+  <si>
+    <t>Revised the flowchart to reflect the actual MVC architecture before adding it to the report.</t>
+  </si>
+  <si>
+    <t>Understand project requirements, generate Java code, explain synchronization concepts and support report writing.</t>
+  </si>
+  <si>
+    <t>Helped understand payroll processing, synchronization mechanisms and speeded up implementation.</t>
+  </si>
+  <si>
+    <t>Review CSV schema, UML design and improve report structure.</t>
+  </si>
+  <si>
+    <t>Provided suggestions for database schema, documentation and presentation content..</t>
+  </si>
+  <si>
+    <t>Code completion and Java programming assistance.</t>
+  </si>
+  <si>
+    <t>Speeded up coding by suggesting Java syntax and reducing repetitive coding.</t>
   </si>
 </sst>
 </file>
@@ -574,41 +759,48 @@
       <sz val="16"/>
       <color rgb="FF2E75B6"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="14"/>
       <color rgb="FF2E75B6"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <i/>
       <sz val="9"/>
       <color rgb="FF666666"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <i/>
       <sz val="10"/>
       <color rgb="FF666666"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="16"/>
       <color rgb="FFFF0000"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -616,26 +808,31 @@
       <sz val="10"/>
       <color rgb="FFFF0000"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="12"/>
       <color rgb="FFFF0000"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <i/>
       <sz val="10"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
@@ -671,7 +868,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -692,6 +889,17 @@
       <bottom style="thin">
         <color rgb="FFCCCCCC"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top/>
+      <bottom/>
       <diagonal/>
     </border>
   </borders>
@@ -735,21 +943,21 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1073,7 +1281,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="22"/>
@@ -1092,7 +1300,7 @@
         <v>2</v>
       </c>
       <c r="C4" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
@@ -1100,7 +1308,7 @@
         <v>3</v>
       </c>
       <c r="C5" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
@@ -1108,7 +1316,7 @@
         <v>4</v>
       </c>
       <c r="C6" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
@@ -1116,7 +1324,7 @@
         <v>5</v>
       </c>
       <c r="C7" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="18" x14ac:dyDescent="0.35">
@@ -1128,8 +1336,8 @@
       <c r="A10" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C10" t="s">
-        <v>121</v>
+      <c r="C10">
+        <v>60</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
@@ -1137,16 +1345,16 @@
         <v>8</v>
       </c>
       <c r="C11" s="3">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C12" s="4" t="e">
+      <c r="C12" s="4">
         <f>C11/C10</f>
-        <v>#VALUE!</v>
+        <v>0.23333333333333334</v>
       </c>
       <c r="E12" s="5" t="s">
         <v>10</v>
@@ -1157,7 +1365,7 @@
         <v>11</v>
       </c>
       <c r="C13" s="3">
-        <v>12</v>
+        <v>8</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="18" x14ac:dyDescent="0.35">
@@ -1179,51 +1387,51 @@
         <v>16</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A17" s="7" t="s">
         <v>17</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>122</v>
+        <v>232</v>
       </c>
       <c r="C17" s="7" t="s">
         <v>18</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A18" s="7" t="s">
         <v>19</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>123</v>
+        <v>234</v>
       </c>
       <c r="C18" s="7" t="s">
         <v>20</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A19" s="7" t="s">
         <v>21</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>22</v>
+        <v>236</v>
       </c>
       <c r="C19" s="7" t="s">
         <v>18</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>23</v>
+        <v>237</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" s="7" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B20" s="7"/>
       <c r="C20" s="7"/>
@@ -1231,62 +1439,62 @@
     </row>
     <row r="22" spans="1:4" ht="18" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C23" s="6" t="s">
         <v>26</v>
-      </c>
-      <c r="B23" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="C23" s="6" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24" s="7" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B24" s="8">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C24" s="9" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25" s="7" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B25" s="8">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C25" s="9" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26" s="7" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B26" s="8">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C26" s="9" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A27" s="7" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B27" s="8">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C27" s="9" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
   </sheetData>
@@ -1312,8 +1520,8 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="23" t="s">
-        <v>34</v>
+      <c r="A1" s="21" t="s">
+        <v>32</v>
       </c>
       <c r="B1" s="22"/>
       <c r="C1" s="22"/>
@@ -1324,8 +1532,8 @@
       <c r="H1" s="22"/>
     </row>
     <row r="2" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="21" t="s">
-        <v>35</v>
+      <c r="A2" s="23" t="s">
+        <v>33</v>
       </c>
       <c r="B2" s="22"/>
       <c r="C2" s="22"/>
@@ -1337,284 +1545,388 @@
     </row>
     <row r="3" spans="1:8" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="C3" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="D3" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="E3" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="F3" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="G3" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="H3" s="6" t="s">
         <v>41</v>
-      </c>
-      <c r="G3" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="H3" s="6" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="100.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="7" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>126</v>
+        <v>116</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>127</v>
+        <v>117</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>128</v>
+        <v>118</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>129</v>
+        <v>119</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>134</v>
-      </c>
-      <c r="H4" s="7" t="s">
-        <v>46</v>
-      </c>
+        <v>124</v>
+      </c>
+      <c r="H4" s="7"/>
     </row>
     <row r="5" spans="1:8" ht="100.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="7" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>131</v>
+        <v>121</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>132</v>
+        <v>122</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>133</v>
+        <v>123</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>135</v>
-      </c>
-      <c r="H5" s="7" t="s">
-        <v>49</v>
-      </c>
+        <v>125</v>
+      </c>
+      <c r="H5" s="7"/>
     </row>
     <row r="6" spans="1:8" ht="100.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="7" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>136</v>
+        <v>126</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>137</v>
+        <v>127</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>138</v>
+        <v>128</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>139</v>
+        <v>129</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>140</v>
-      </c>
-      <c r="H6" s="7" t="s">
-        <v>52</v>
-      </c>
+        <v>130</v>
+      </c>
+      <c r="H6" s="7"/>
     </row>
     <row r="7" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="18" t="s">
+      <c r="A7" s="20" t="s">
+        <v>170</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>133</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>134</v>
+      </c>
+      <c r="G7" s="7" t="s">
+        <v>135</v>
+      </c>
+      <c r="H7" s="7"/>
+    </row>
+    <row r="8" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="20" t="s">
+        <v>171</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="D8" s="19" t="s">
+        <v>145</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>142</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>143</v>
+      </c>
+      <c r="G8" s="18" t="s">
+        <v>144</v>
+      </c>
+      <c r="H8" s="7"/>
+    </row>
+    <row r="9" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="20" t="s">
+        <v>172</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>146</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>147</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>148</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>149</v>
+      </c>
+      <c r="G9" s="7" t="s">
+        <v>150</v>
+      </c>
+      <c r="H9" s="7"/>
+    </row>
+    <row r="10" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="20" t="s">
+        <v>173</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="C10" s="7" t="s">
         <v>151</v>
       </c>
-      <c r="B7" s="7" t="s">
-        <v>51</v>
-      </c>
-      <c r="C7" s="7" t="s">
-        <v>141</v>
-      </c>
-      <c r="D7" s="7" t="s">
-        <v>142</v>
-      </c>
-      <c r="E7" s="7" t="s">
-        <v>143</v>
-      </c>
-      <c r="F7" s="7" t="s">
-        <v>144</v>
-      </c>
-      <c r="G7" s="7" t="s">
-        <v>145</v>
-      </c>
-      <c r="H7" s="7"/>
-    </row>
-    <row r="8" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="18" t="s">
+      <c r="D10" s="7" t="s">
         <v>152</v>
       </c>
-      <c r="B8" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="C8" s="7" t="s">
+      <c r="E10" s="7" t="s">
         <v>153</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="F10" s="7" t="s">
         <v>154</v>
       </c>
-      <c r="E8" s="7" t="s">
+      <c r="G10" s="18" t="s">
         <v>155</v>
       </c>
-      <c r="F8" s="7" t="s">
+      <c r="H10" s="7"/>
+    </row>
+    <row r="11" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="20" t="s">
+        <v>174</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>151</v>
+      </c>
+      <c r="D11" s="7" t="s">
         <v>156</v>
       </c>
-      <c r="G8" s="20" t="s">
+      <c r="E11" s="7" t="s">
+        <v>157</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>158</v>
+      </c>
+      <c r="G11" s="7" t="s">
+        <v>159</v>
+      </c>
+      <c r="H11" s="7"/>
+    </row>
+    <row r="12" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="20" t="s">
+        <v>175</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>162</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>164</v>
+      </c>
+      <c r="F12" s="7" t="s">
+        <v>166</v>
+      </c>
+      <c r="G12" s="7" t="s">
+        <v>168</v>
+      </c>
+      <c r="H12" s="7"/>
+    </row>
+    <row r="13" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="20" t="s">
+        <v>176</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="C13" s="7" t="s">
         <v>161</v>
       </c>
-      <c r="H8" s="7" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="18" t="s">
-        <v>164</v>
-      </c>
-      <c r="B9" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="C9" s="7" t="s">
-        <v>166</v>
-      </c>
-      <c r="D9" s="7" t="s">
-        <v>168</v>
-      </c>
-      <c r="E9" s="7" t="s">
-        <v>159</v>
-      </c>
-      <c r="F9" s="7" t="s">
-        <v>157</v>
-      </c>
-      <c r="G9" s="19" t="s">
-        <v>162</v>
-      </c>
-      <c r="H9" s="7"/>
-    </row>
-    <row r="10" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="18" t="s">
+      <c r="D13" s="7" t="s">
+        <v>163</v>
+      </c>
+      <c r="E13" s="7" t="s">
         <v>165</v>
       </c>
-      <c r="B10" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="C10" s="7" t="s">
+      <c r="F13" s="7" t="s">
         <v>167</v>
       </c>
-      <c r="D10" s="7" t="s">
+      <c r="G13" s="7" t="s">
         <v>169</v>
       </c>
-      <c r="E10" s="7" t="s">
-        <v>160</v>
-      </c>
-      <c r="F10" s="7" t="s">
-        <v>158</v>
-      </c>
-      <c r="G10" s="19" t="s">
-        <v>163</v>
-      </c>
-      <c r="H10" s="7"/>
-    </row>
-    <row r="11" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="7"/>
-      <c r="B11" s="7"/>
-      <c r="C11" s="7"/>
-      <c r="D11" s="7"/>
-      <c r="E11" s="7"/>
-      <c r="F11" s="7"/>
-      <c r="G11" s="7"/>
-      <c r="H11" s="7"/>
-    </row>
-    <row r="12" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="7"/>
-      <c r="B12" s="7"/>
-      <c r="C12" s="7"/>
-      <c r="D12" s="7"/>
-      <c r="E12" s="7"/>
-      <c r="F12" s="7"/>
-      <c r="G12" s="7"/>
-      <c r="H12" s="7"/>
-    </row>
-    <row r="13" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="7"/>
-      <c r="B13" s="7"/>
-      <c r="C13" s="7"/>
-      <c r="D13" s="7"/>
-      <c r="E13" s="7"/>
-      <c r="F13" s="7"/>
-      <c r="G13" s="7"/>
       <c r="H13" s="7"/>
     </row>
     <row r="14" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="7"/>
-      <c r="B14" s="7"/>
-      <c r="C14" s="7"/>
-      <c r="D14" s="7"/>
-      <c r="E14" s="7"/>
-      <c r="F14" s="7"/>
-      <c r="G14" s="7"/>
+      <c r="A14" s="20" t="s">
+        <v>195</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>196</v>
+      </c>
+      <c r="D14" s="7" t="s">
+        <v>197</v>
+      </c>
+      <c r="E14" s="7" t="s">
+        <v>198</v>
+      </c>
+      <c r="F14" s="7" t="s">
+        <v>199</v>
+      </c>
+      <c r="G14" s="7" t="s">
+        <v>212</v>
+      </c>
       <c r="H14" s="7"/>
     </row>
     <row r="15" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="7"/>
-      <c r="B15" s="7"/>
-      <c r="C15" s="7"/>
-      <c r="D15" s="7"/>
-      <c r="E15" s="7"/>
-      <c r="F15" s="7"/>
-      <c r="G15" s="7"/>
+      <c r="A15" s="20" t="s">
+        <v>216</v>
+      </c>
+      <c r="B15" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C15" s="7" t="s">
+        <v>200</v>
+      </c>
+      <c r="D15" s="7" t="s">
+        <v>201</v>
+      </c>
+      <c r="E15" s="7" t="s">
+        <v>202</v>
+      </c>
+      <c r="F15" s="7" t="s">
+        <v>203</v>
+      </c>
+      <c r="G15" s="7" t="s">
+        <v>213</v>
+      </c>
       <c r="H15" s="7"/>
     </row>
     <row r="16" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="7"/>
-      <c r="B16" s="7"/>
-      <c r="C16" s="7"/>
-      <c r="D16" s="7"/>
-      <c r="E16" s="7"/>
-      <c r="F16" s="7"/>
-      <c r="G16" s="7"/>
+      <c r="A16" s="20" t="s">
+        <v>217</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>204</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>205</v>
+      </c>
+      <c r="E16" s="7" t="s">
+        <v>206</v>
+      </c>
+      <c r="F16" s="7" t="s">
+        <v>207</v>
+      </c>
+      <c r="G16" s="7" t="s">
+        <v>214</v>
+      </c>
       <c r="H16" s="7"/>
     </row>
     <row r="17" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="7"/>
-      <c r="B17" s="7"/>
-      <c r="C17" s="7"/>
-      <c r="D17" s="7"/>
-      <c r="E17" s="7"/>
-      <c r="F17" s="7"/>
-      <c r="G17" s="7"/>
+      <c r="A17" s="20" t="s">
+        <v>218</v>
+      </c>
+      <c r="B17" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C17" s="7" t="s">
+        <v>208</v>
+      </c>
+      <c r="D17" s="7" t="s">
+        <v>209</v>
+      </c>
+      <c r="E17" s="7" t="s">
+        <v>210</v>
+      </c>
+      <c r="F17" s="7" t="s">
+        <v>211</v>
+      </c>
+      <c r="G17" s="7" t="s">
+        <v>215</v>
+      </c>
       <c r="H17" s="7"/>
     </row>
     <row r="18" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="7"/>
-      <c r="B18" s="7"/>
-      <c r="C18" s="7"/>
-      <c r="D18" s="7"/>
-      <c r="E18" s="7"/>
-      <c r="F18" s="7"/>
-      <c r="G18" s="7"/>
+      <c r="A18" s="20" t="s">
+        <v>219</v>
+      </c>
+      <c r="B18" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="C18" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="E18" s="7" t="s">
+        <v>222</v>
+      </c>
+      <c r="F18" s="7" t="s">
+        <v>223</v>
+      </c>
+      <c r="G18" s="7" t="s">
+        <v>223</v>
+      </c>
       <c r="H18" s="7"/>
     </row>
     <row r="19" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1718,7 +2030,7 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="25" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="B1" s="22"/>
       <c r="C1" s="22"/>
@@ -1728,7 +2040,7 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="24" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="B2" s="22"/>
       <c r="C2" s="22"/>
@@ -1738,47 +2050,47 @@
     </row>
     <row r="3" spans="1:6" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="F3" s="6" t="s">
         <v>55</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="C3" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="D3" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="E3" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="F3" s="6" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="7" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="7" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B5" s="7"/>
       <c r="C5" s="7"/>
@@ -1787,84 +2099,144 @@
       <c r="F5" s="7"/>
     </row>
     <row r="6" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="18" t="s">
-        <v>151</v>
+      <c r="A6" s="20" t="s">
+        <v>170</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>146</v>
+        <v>136</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>147</v>
+        <v>137</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>149</v>
+        <v>139</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>150</v>
+        <v>140</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="18" t="s">
-        <v>152</v>
+      <c r="A7" s="20" t="s">
+        <v>177</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>171</v>
+        <v>136</v>
       </c>
       <c r="C7" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="20" t="s">
         <v>172</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="B8" s="7" t="s">
+        <v>182</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>183</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>184</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="20" t="s">
         <v>173</v>
       </c>
-      <c r="E7" s="7" t="s">
-        <v>174</v>
-      </c>
-      <c r="F7" s="7" t="s">
+      <c r="B9" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>187</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>188</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>189</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="20" t="s">
         <v>175</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="7"/>
-      <c r="B8" s="7"/>
-      <c r="C8" s="7"/>
-      <c r="D8" s="7"/>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7"/>
-    </row>
-    <row r="9" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="7"/>
-      <c r="B9" s="7"/>
-      <c r="C9" s="7"/>
-      <c r="D9" s="7"/>
-      <c r="E9" s="7"/>
-      <c r="F9" s="7"/>
-    </row>
-    <row r="10" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="7"/>
-      <c r="B10" s="7"/>
-      <c r="C10" s="7"/>
-      <c r="D10" s="7"/>
-      <c r="E10" s="7"/>
-      <c r="F10" s="7"/>
+      <c r="B10" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>191</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>193</v>
+      </c>
+      <c r="F10" s="7" t="s">
+        <v>194</v>
+      </c>
     </row>
     <row r="11" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="7"/>
-      <c r="B11" s="7"/>
-      <c r="C11" s="7"/>
-      <c r="D11" s="7"/>
-      <c r="E11" s="7"/>
-      <c r="F11" s="7"/>
+      <c r="A11" s="20" t="s">
+        <v>176</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>224</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>225</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>226</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>227</v>
+      </c>
     </row>
     <row r="12" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="7"/>
-      <c r="B12" s="7"/>
-      <c r="C12" s="7"/>
-      <c r="D12" s="7"/>
-      <c r="E12" s="7"/>
-      <c r="F12" s="7"/>
+      <c r="A12" s="20" t="s">
+        <v>195</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>228</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>230</v>
+      </c>
+      <c r="F12" s="7" t="s">
+        <v>231</v>
+      </c>
     </row>
     <row r="13" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="7"/>
@@ -1964,73 +2336,73 @@
     </row>
     <row r="30" spans="1:6" ht="18" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" s="10" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="B31" s="10" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="C31" s="10" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
     </row>
     <row r="32" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A32" s="7" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="B32" s="7" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="C32" s="7" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
     </row>
     <row r="33" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A33" s="7" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="B33" s="7" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A34" s="7" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="B34" s="7" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="C34" s="7" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
     </row>
     <row r="35" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A35" s="7" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="B35" s="7" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="C35" s="7" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
     </row>
     <row r="36" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A36" s="7" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="B36" s="7" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="C36" s="7" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
     </row>
   </sheetData>
@@ -2054,8 +2426,8 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" s="23" t="s">
-        <v>84</v>
+      <c r="A1" s="21" t="s">
+        <v>79</v>
       </c>
       <c r="B1" s="22"/>
       <c r="C1" s="22"/>
@@ -2063,7 +2435,7 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="26" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="B2" s="22"/>
       <c r="C2" s="22"/>
@@ -2071,204 +2443,204 @@
     </row>
     <row r="4" spans="1:4" ht="18" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="6" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="12" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="D6" s="13"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="12" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="D7" s="13"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="12" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="D8" s="13"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="12" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="D9" s="13"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" s="12" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="D10" s="13"/>
     </row>
     <row r="12" spans="1:4" ht="18" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" s="6" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="D13" s="11" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" s="12" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="C14" s="12" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="D14" s="13"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" s="12" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="C15" s="12" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="D15" s="13"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" s="12" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="C16" s="12" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="D16" s="13"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" s="12" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="D17" s="13"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" s="12" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="B18" s="13" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="C18" s="12" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="D18" s="13"/>
     </row>
     <row r="20" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A20" s="14" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" s="15" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" s="15" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
     </row>
     <row r="25" spans="1:4" ht="18" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26" s="16" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
     </row>
     <row r="27" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A27" s="17" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B27" s="10" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="D27" s="10" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A28" s="9" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B28" s="7"/>
       <c r="C28" s="7"/>
@@ -2276,7 +2648,7 @@
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29" s="9" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="B29" s="7"/>
       <c r="C29" s="7"/>
@@ -2284,7 +2656,7 @@
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A30" s="9" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="B30" s="7"/>
       <c r="C30" s="7"/>

</xml_diff>